<commit_message>
Provenance: require lot codes on primary packaging, not secondary
</commit_message>
<xml_diff>
--- a/public/samples/westridge-delivery-note.xlsx
+++ b/public/samples/westridge-delivery-note.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -641,112 +641,135 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Double Cream</v>
+        <v>500ml Retail Tub</v>
       </c>
       <c r="B20" t="str">
-        <v>HF-070926-C</v>
+        <v/>
       </c>
       <c r="C20" t="str">
-        <v>400</v>
+        <v>5000</v>
       </c>
       <c r="D20" t="str">
-        <v>kg</v>
+        <v>ea</v>
       </c>
       <c r="E20" t="str">
-        <v>14 Sep 2026</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v>3.1</v>
+        <v/>
       </c>
       <c r="G20" t="str">
-        <v>10L</v>
+        <v>Sleeve of 50</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Hazelnut Praline Paste</v>
+        <v>Double Cream</v>
       </c>
       <c r="B21" t="str">
-        <v>HP-2609-01</v>
+        <v>HF-070926-C</v>
       </c>
       <c r="C21" t="str">
-        <v>15</v>
+        <v>400</v>
       </c>
       <c r="D21" t="str">
         <v>kg</v>
       </c>
       <c r="E21" t="str">
-        <v>02 Mar 2027</v>
+        <v>14 Sep 2026</v>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>3.1</v>
       </c>
       <c r="G21" t="str">
-        <v>5kg</v>
+        <v>10L</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Whole Milk</v>
+        <v>Hazelnut Praline Paste</v>
       </c>
       <c r="B22" t="str">
-        <v>HF-070926</v>
+        <v>HP-2609-01</v>
       </c>
       <c r="C22" t="str">
-        <v>18500</v>
+        <v>15</v>
       </c>
       <c r="D22" t="str">
-        <v>L</v>
+        <v>kg</v>
       </c>
       <c r="E22" t="str">
-        <v>11 Sep 2026</v>
+        <v>02 Mar 2027</v>
       </c>
       <c r="F22" t="str">
-        <v>3.4</v>
+        <v/>
       </c>
       <c r="G22" t="str">
-        <v>Bulk tanker</v>
+        <v>5kg</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>Whole Milk</v>
+      </c>
+      <c r="B23" t="str">
+        <v>HF-070926</v>
+      </c>
+      <c r="C23" t="str">
+        <v>18500</v>
+      </c>
+      <c r="D23" t="str">
+        <v>L</v>
+      </c>
+      <c r="E23" t="str">
+        <v>11 Sep 2026</v>
+      </c>
+      <c r="F23" t="str">
+        <v>3.4</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Bulk tanker</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B23" t="str">
-        <v/>
-      </c>
-      <c r="C23" t="str">
-        <v>20820</v>
-      </c>
-      <c r="D23" t="str">
-        <v/>
-      </c>
-      <c r="E23" t="str">
-        <v/>
-      </c>
-      <c r="F23" t="str">
-        <v/>
-      </c>
-      <c r="G23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Received by:</v>
-      </c>
-      <c r="B25" t="str">
-        <v/>
-      </c>
-      <c r="D25" t="str">
-        <v>Signature:</v>
-      </c>
-      <c r="E25" t="str">
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v>25820</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>Received by:</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v>Signature:</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>All goods remain the property of Westridge Food Ingredients Ltd until paid for in full.</v>
       </c>
     </row>
@@ -758,7 +781,7 @@
     <mergeCell ref="A5:C5"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>